<commit_message>
Add ELIIY Power suppliers, partners and shareholders tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NvsxtgCjxqSPqHvgLtoBEU
</commit_message>
<xml_diff>
--- a/Eliiy_Power_Products_India_China_Rates.xlsx
+++ b/Eliiy_Power_Products_India_China_Rates.xlsx
@@ -13,10 +13,11 @@
     <sheet name="Product Photos" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Product Specs" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Where Used" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Price Comparison" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Market Benchmarks" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Sources" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="How Prices Were Got" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Suppliers &amp; Partners" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Price Comparison" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Market Benchmarks" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Sources" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="How Prices Were Got" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="719">
   <si>
     <t xml:space="preserve">ELIIY Power (Japan) – Product, Application &amp; Cost Benchmark</t>
   </si>
@@ -1011,6 +1012,453 @@
     <t xml:space="preserve">S42</t>
   </si>
   <si>
+    <t xml:space="preserve">ELIIY Power – Suppliers, Partners &amp; Shareholders (public sources)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Researched 27 Oct 2026. ELIIY is private and publishes no supplier list – each row is backed by a patent, press release or report. Green = confirmed, yellow = partial / historical.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What they supply / do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sumitomo Osaka Cement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LFP (lithium iron phosphate) cathode material – newly developed grade adopted by ELIIY; cathode jointly optimised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIIY press release says its cathode uses LFP developed by Sumitomo Osaka Cement; co-applicant on cathode patent US 2013/0266843</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2010 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.eliiypower.co.jp/files/pdf/20101224.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nagano Automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell manufacturing / assembly equipment (electrode-assembly and secondary-battery production apparatus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-assignee on 3 US manufacturing-process patents: 9,450,268; 9,853,329; 9,871,268</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2014–2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://patents.justia.com/assignee/eliiy-power-co-ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UBE (Ube Industries)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrolyte – high-temperature, ignition-resistant electrolyte development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three-way joint development with Mazda and ELIIY on 12 V Li-ion car starter battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed (dev.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.themachinist.in/news/4181/mazda-eliiy-power-ube-industries-enter-agreement/page/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toray Industries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shareholder; separator maker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World #2 battery separator producer. Bought most of Sharp's stake in 2013 via Toray Battery Separator Film. Separator supply likely but not publicly confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japanese Wikipedia (shareholding history); INITIAL shareholder list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2013 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ja.wikipedia.org/wiki/%E3%82%A8%E3%83%AA%E3%83%BC%E3%83%91%E3%83%AF%E3%83%BC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dai Nippon Printing (DNP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shareholder; process partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helped solve electrode-coating problem in early L2 project; DNP also makes Li-ion pouch film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japanese Wikipedia; listed in ELIIY 2010 shareholder table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2004 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honda Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OEM customer / co-developer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-developed motorcycle starter battery casing &amp; sealing; buys HY85S / HY93-C / HY110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-assignee on US patents 10,818,887 and 11,502,339</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2017 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suzuki Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largest shareholder; OEM customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¥10 bn equity + ¥15 bn convertible bonds (Nov 2023) → 21.59%; joint development of large Li-ion for ESS and mobility; buys HY93SS / HY110SS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIIY / Suzuki press release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2012 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.eliiypower.co.jp/files/pdf/20231114.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daiwa House Industry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shareholder; channel partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.01% (via Enesarb) as of Nov 2023; sells ELIIY ESS in homes, rentals, commercial &amp; logistics buildings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suzuki release; Japanese Wikipedia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2006 →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mazda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-developer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 V Li-ion car starter battery (with UBE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint development agreement, Mar 2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuji Electric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charge/discharge control (PCS) for container system using ELIIY battery at NITE Osaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newswitch article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed (project)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://newswitch.jp/p/4756</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enphase Energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell-pack customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8-cell 1.2 kWh modules + BMU for Enphase AC Battery, 6-yr deal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIIY press release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2015–2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.eliiypower.co.jp/files/english/pdf/20151016_Release.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NTN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultra-compact EV using ELIIY cells (Kuwana demo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://newswitch.jp/p/1467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alps Alpine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shareholder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role not disclosed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INITIAL shareholder list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://initial.inc/companies/A-04762</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~20 Kawasaki local firms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabrication suppliers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storage-unit frames, battery-system development; ≈¥300 m orders in FY2011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kawasaki City committee document (2012)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY2011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.city.kawasaki.jp/980/cmsfiles/contents/0000042/42584/241031shimin1-1.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sharp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Former shareholder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Major shareholder 2008–2013, stake sold to Toray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japanese Wikipedia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2008–13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plant facts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cells made in-house at Kawasaki (P and L plants), fully automated stack-type line: kneading → coating → drying/pressing → cutting → stacking → case welding → electrolyte fill → formation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Capacity: 200k cells/yr (2010) → 1.0 m (2012) → planned 1.7 m after Enphase expansion (2015). Approx. 1.7 m × 155 Wh ≈ 0.26 GWh/yr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Paid-in capital ≈ ¥50.2 bn (Nov 2023); employees 101–500.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still unknown – how to fill the gaps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost / access</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anode (graphite), separator, foil, case, BMS IC suppliers</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Teikoku Databank (TDB) or Tokyo Shoko Research (TSR) full company report – lists </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">主要仕入先 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(main suppliers) and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">主要販売先</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid; order via tdb.co.jp / tsr-net.co.jp or D&amp;B India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imports from China / Korea to ELIIY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volza / Panjiva consignee search 'ELIIY POWER' (China &amp; Korea export records)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid subscription; free web search returned no records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Components inside products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teardown of HY93-C or POWER YIILE 3 – read IC, connector, resin and PCS markings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One product purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full patent co-applicant list</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">J-PlatPat search </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">出願人 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">エリーパワー </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Japanese filings are far more numerous than US)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Free – j-platpat.inpit.go.jp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct confirmation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIIY contact form; Battery Japan / Smart Energy Week, Tokyo Big Sight (Feb–Mar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free</t>
+  </si>
+  <si>
     <t xml:space="preserve">ELIIY Power vs Indian OEM vs Chinese OEM – Rates</t>
   </si>
   <si>
@@ -1578,9 +2026,6 @@
     <t xml:space="preserve">Enphase battery-pack supply deal (Oct 2015)</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.eliiypower.co.jp/files/english/pdf/20151016_Release.pdf</t>
-  </si>
-  <si>
     <t xml:space="preserve">S19</t>
   </si>
   <si>
@@ -1765,9 +2210,6 @@
   </si>
   <si>
     <t xml:space="preserve">Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence</t>
   </si>
   <si>
     <t xml:space="preserve">ELIIY prices</t>
@@ -1845,7 +2287,7 @@
     <numFmt numFmtId="171" formatCode="#,##0"/>
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1965,6 +2407,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="9"/>
       <name val="Arial"/>
@@ -1992,7 +2440,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2014,7 +2462,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -2067,7 +2521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2156,6 +2610,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2180,7 +2638,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2257,7 +2715,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -2523,11 +2981,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="56606757"/>
-        <c:axId val="17746005"/>
+        <c:axId val="75320587"/>
+        <c:axId val="18561436"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="56606757"/>
+        <c:axId val="75320587"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2559,7 +3017,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17746005"/>
+        <c:crossAx val="18561436"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2567,7 +3025,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17746005"/>
+        <c:axId val="18561436"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2633,7 +3091,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56606757"/>
+        <c:crossAx val="75320587"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3102,6 +3560,134 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
+        <v>697</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>698</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>702</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>703</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>705</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>710</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>711</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36" t="s">
+        <v>714</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>715</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>718</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -4885,6 +5471,568 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>394</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>394</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>424</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12" t="s">
+        <v>430</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>431</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="181.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="125.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H5" r:id="rId1" display="https://www.eliiypower.co.jp/files/pdf/20101224.pdf"/>
+    <hyperlink ref="H6" r:id="rId2" display="https://patents.justia.com/assignee/eliiy-power-co-ltd"/>
+    <hyperlink ref="H7" r:id="rId3" display="https://www.themachinist.in/news/4181/mazda-eliiy-power-ube-industries-enter-agreement/page/2"/>
+    <hyperlink ref="H8" r:id="rId4" display="https://ja.wikipedia.org/wiki/%E3%82%A8%E3%83%AA%E3%83%BC%E3%83%91%E3%83%AF%E3%83%BC"/>
+    <hyperlink ref="H9" r:id="rId5" display="https://ja.wikipedia.org/wiki/%E3%82%A8%E3%83%AA%E3%83%BC%E3%83%91%E3%83%AF%E3%83%BC"/>
+    <hyperlink ref="H10" r:id="rId6" display="https://patents.justia.com/assignee/eliiy-power-co-ltd"/>
+    <hyperlink ref="H11" r:id="rId7" display="https://www.eliiypower.co.jp/files/pdf/20231114.pdf"/>
+    <hyperlink ref="H12" r:id="rId8" display="https://www.eliiypower.co.jp/files/pdf/20231114.pdf"/>
+    <hyperlink ref="H13" r:id="rId9" display="https://www.themachinist.in/news/4181/mazda-eliiy-power-ube-industries-enter-agreement/page/2"/>
+    <hyperlink ref="H14" r:id="rId10" display="https://newswitch.jp/p/4756"/>
+    <hyperlink ref="H15" r:id="rId11" display="https://www.eliiypower.co.jp/files/english/pdf/20151016_Release.pdf"/>
+    <hyperlink ref="H16" r:id="rId12" display="https://newswitch.jp/p/1467"/>
+    <hyperlink ref="H17" r:id="rId13" display="https://initial.inc/companies/A-04762"/>
+    <hyperlink ref="H18" r:id="rId14" display="https://www.city.kawasaki.jp/980/cmsfiles/contents/0000042/42584/241031shimin1-1.pdf"/>
+    <hyperlink ref="H19" r:id="rId15" display="https://ja.wikipedia.org/wiki/%E3%82%A8%E3%83%AA%E3%83%BC%E3%83%91%E3%83%AF%E3%83%BC"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Z29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4912,12 +6060,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>327</v>
+        <v>448</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>328</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4928,76 +6076,76 @@
         <v>61</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>329</v>
+        <v>450</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>330</v>
+        <v>451</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>331</v>
+        <v>452</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>332</v>
+        <v>453</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>333</v>
+        <v>454</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>334</v>
+        <v>455</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>335</v>
+        <v>456</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>336</v>
+        <v>457</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>337</v>
+        <v>458</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>338</v>
+        <v>459</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>339</v>
+        <v>460</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>340</v>
+        <v>461</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>341</v>
+        <v>462</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>342</v>
+        <v>463</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>343</v>
+        <v>464</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>344</v>
+        <v>465</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>345</v>
+        <v>466</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>346</v>
+        <v>467</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>347</v>
+        <v>468</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>348</v>
+        <v>469</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>349</v>
+        <v>470</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>350</v>
+        <v>471</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>351</v>
+        <v>472</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>352</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5005,87 +6153,87 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>353</v>
+        <v>474</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="23" t="n">
         <v>0.054</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <v>37790</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="H5" s="25" t="n">
+        <v>475</v>
+      </c>
+      <c r="H5" s="26" t="n">
         <f aca="false">IF(E5="","Quote only",E5*INDEX(Assumptions!$B$12:$B$16,MATCH(F5,Assumptions!$A$12:$A$16,0)))</f>
         <v>23067.016</v>
       </c>
-      <c r="I5" s="25" t="n">
+      <c r="I5" s="26" t="n">
         <f aca="false">IF(ISNUMBER(H5),H5/D5,"–")</f>
         <v>427166.962962963</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="K5" s="23" t="n">
+        <v>476</v>
+      </c>
+      <c r="K5" s="24" t="n">
         <v>1386</v>
       </c>
-      <c r="L5" s="23" t="n">
+      <c r="L5" s="24" t="n">
         <v>1690</v>
       </c>
-      <c r="M5" s="24" t="s">
+      <c r="M5" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N5" s="25" t="n">
+      <c r="N5" s="26" t="n">
         <f aca="false">AVERAGE(K5:L5)*INDEX(Assumptions!$B$12:$B$16,MATCH(M5,Assumptions!$A$12:$A$16,0))</f>
         <v>1538</v>
       </c>
-      <c r="O5" s="25" t="n">
+      <c r="O5" s="26" t="n">
         <f aca="false">N5/D5</f>
         <v>28481.4814814815</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>356</v>
+        <v>477</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="R5" s="26" t="n">
+        <v>478</v>
+      </c>
+      <c r="R5" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="S5" s="26" t="n">
+      <c r="S5" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="T5" s="24" t="s">
+      <c r="T5" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="U5" s="25" t="n">
+      <c r="U5" s="26" t="n">
         <f aca="false">AVERAGE(R5:S5)*INDEX(Assumptions!$B$12:$B$16,MATCH(T5,Assumptions!$A$12:$A$16,0))</f>
         <v>1935.6</v>
       </c>
-      <c r="V5" s="25" t="n">
+      <c r="V5" s="26" t="n">
         <f aca="false">U5/D5</f>
         <v>35844.4444444444</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>358</v>
-      </c>
-      <c r="X5" s="27" t="n">
+        <v>479</v>
+      </c>
+      <c r="X5" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H5),H5/U5,"–")</f>
         <v>11.9172432320727</v>
       </c>
-      <c r="Y5" s="27" t="n">
+      <c r="Y5" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H5),H5/N5,"–")</f>
         <v>14.9980598179454</v>
       </c>
       <c r="Z5" s="6" t="s">
-        <v>359</v>
+        <v>480</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5093,87 +6241,87 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>360</v>
+        <v>481</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="23" t="n">
         <v>0.072</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <v>44460</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="H6" s="25" t="n">
+        <v>475</v>
+      </c>
+      <c r="H6" s="26" t="n">
         <f aca="false">IF(E6="","Quote only",E6*INDEX(Assumptions!$B$12:$B$16,MATCH(F6,Assumptions!$A$12:$A$16,0)))</f>
         <v>27138.384</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="I6" s="26" t="n">
         <f aca="false">IF(ISNUMBER(H6),H6/D6,"–")</f>
         <v>376922</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>361</v>
-      </c>
-      <c r="K6" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="K6" s="24" t="n">
         <v>1800</v>
       </c>
-      <c r="L6" s="23" t="n">
+      <c r="L6" s="24" t="n">
         <v>2045</v>
       </c>
-      <c r="M6" s="24" t="s">
+      <c r="M6" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N6" s="25" t="n">
+      <c r="N6" s="26" t="n">
         <f aca="false">AVERAGE(K6:L6)*INDEX(Assumptions!$B$12:$B$16,MATCH(M6,Assumptions!$A$12:$A$16,0))</f>
         <v>1922.5</v>
       </c>
-      <c r="O6" s="25" t="n">
+      <c r="O6" s="26" t="n">
         <f aca="false">N6/D6</f>
         <v>26701.3888888889</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>362</v>
+        <v>483</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>363</v>
-      </c>
-      <c r="R6" s="26" t="n">
+        <v>484</v>
+      </c>
+      <c r="R6" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="S6" s="26" t="n">
+      <c r="S6" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="T6" s="24" t="s">
+      <c r="T6" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="U6" s="25" t="n">
+      <c r="U6" s="26" t="n">
         <f aca="false">AVERAGE(R6:S6)*INDEX(Assumptions!$B$12:$B$16,MATCH(T6,Assumptions!$A$12:$A$16,0))</f>
         <v>2661.45</v>
       </c>
-      <c r="V6" s="25" t="n">
+      <c r="V6" s="26" t="n">
         <f aca="false">U6/D6</f>
         <v>36964.5833333333</v>
       </c>
       <c r="W6" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="X6" s="27" t="n">
+        <v>485</v>
+      </c>
+      <c r="X6" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H6),H6/U6,"–")</f>
         <v>10.1968415713239</v>
       </c>
-      <c r="Y6" s="27" t="n">
+      <c r="Y6" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H6),H6/N6,"–")</f>
         <v>14.1161945383615</v>
       </c>
       <c r="Z6" s="6" t="s">
-        <v>359</v>
+        <v>480</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5181,87 +6329,87 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>365</v>
+        <v>486</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>2.5</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <v>1097800</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>366</v>
-      </c>
-      <c r="H7" s="25" t="n">
+        <v>487</v>
+      </c>
+      <c r="H7" s="26" t="n">
         <f aca="false">IF(E7="","Quote only",E7*INDEX(Assumptions!$B$12:$B$16,MATCH(F7,Assumptions!$A$12:$A$16,0)))</f>
         <v>670097.12</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="I7" s="26" t="n">
         <f aca="false">IF(ISNUMBER(H7),H7/D7,"–")</f>
         <v>268038.848</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>367</v>
-      </c>
-      <c r="K7" s="23" t="n">
+        <v>488</v>
+      </c>
+      <c r="K7" s="24" t="n">
         <v>40000</v>
       </c>
-      <c r="L7" s="23" t="n">
+      <c r="L7" s="24" t="n">
         <v>65000</v>
       </c>
-      <c r="M7" s="24" t="s">
+      <c r="M7" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N7" s="25" t="n">
+      <c r="N7" s="26" t="n">
         <f aca="false">AVERAGE(K7:L7)*INDEX(Assumptions!$B$12:$B$16,MATCH(M7,Assumptions!$A$12:$A$16,0))</f>
         <v>52500</v>
       </c>
-      <c r="O7" s="25" t="n">
+      <c r="O7" s="26" t="n">
         <f aca="false">N7/D7</f>
         <v>21000</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>368</v>
+        <v>489</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="R7" s="26" t="n">
+        <v>490</v>
+      </c>
+      <c r="R7" s="27" t="n">
         <v>375</v>
       </c>
-      <c r="S7" s="26" t="n">
+      <c r="S7" s="27" t="n">
         <v>625</v>
       </c>
-      <c r="T7" s="24" t="s">
+      <c r="T7" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="U7" s="25" t="n">
+      <c r="U7" s="26" t="n">
         <f aca="false">AVERAGE(R7:S7)*INDEX(Assumptions!$B$12:$B$16,MATCH(T7,Assumptions!$A$12:$A$16,0))</f>
         <v>48390</v>
       </c>
-      <c r="V7" s="25" t="n">
+      <c r="V7" s="26" t="n">
         <f aca="false">U7/D7</f>
         <v>19356</v>
       </c>
       <c r="W7" s="14" t="s">
-        <v>370</v>
-      </c>
-      <c r="X7" s="27" t="n">
+        <v>491</v>
+      </c>
+      <c r="X7" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H7),H7/U7,"–")</f>
         <v>13.8478429427568</v>
       </c>
-      <c r="Y7" s="27" t="n">
+      <c r="Y7" s="28" t="n">
         <f aca="false">IF(ISNUMBER(H7),H7/N7,"–")</f>
         <v>12.7637546666667</v>
       </c>
       <c r="Z7" s="6" t="s">
-        <v>371</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5269,85 +6417,85 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>372</v>
+        <v>493</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>1.3</v>
       </c>
-      <c r="E8" s="23"/>
-      <c r="F8" s="24" t="s">
+      <c r="E8" s="24"/>
+      <c r="F8" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="H8" s="25" t="str">
+        <v>494</v>
+      </c>
+      <c r="H8" s="26" t="str">
         <f aca="false">IF(E8="","Quote only",E8*INDEX(Assumptions!$B$12:$B$16,MATCH(F8,Assumptions!$A$12:$A$16,0)))</f>
         <v>Quote only</v>
       </c>
-      <c r="I8" s="25" t="str">
+      <c r="I8" s="26" t="str">
         <f aca="false">IF(ISNUMBER(H8),H8/D8,"–")</f>
         <v>–</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>374</v>
-      </c>
-      <c r="K8" s="26" t="n">
+        <v>495</v>
+      </c>
+      <c r="K8" s="27" t="n">
         <v>26000</v>
       </c>
-      <c r="L8" s="26" t="n">
+      <c r="L8" s="27" t="n">
         <v>45500</v>
       </c>
-      <c r="M8" s="24" t="s">
+      <c r="M8" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N8" s="25" t="n">
+      <c r="N8" s="26" t="n">
         <f aca="false">AVERAGE(K8:L8)*INDEX(Assumptions!$B$12:$B$16,MATCH(M8,Assumptions!$A$12:$A$16,0))</f>
         <v>35750</v>
       </c>
-      <c r="O8" s="25" t="n">
+      <c r="O8" s="26" t="n">
         <f aca="false">N8/D8</f>
         <v>27500</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>375</v>
+        <v>496</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="R8" s="26" t="n">
+        <v>497</v>
+      </c>
+      <c r="R8" s="27" t="n">
         <v>180</v>
       </c>
-      <c r="S8" s="26" t="n">
+      <c r="S8" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="T8" s="24" t="s">
+      <c r="T8" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="U8" s="25" t="n">
+      <c r="U8" s="26" t="n">
         <f aca="false">AVERAGE(R8:S8)*INDEX(Assumptions!$B$12:$B$16,MATCH(T8,Assumptions!$A$12:$A$16,0))</f>
         <v>23227.2</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="26" t="n">
         <f aca="false">U8/D8</f>
         <v>17867.0769230769</v>
       </c>
       <c r="W8" s="14" t="s">
-        <v>377</v>
-      </c>
-      <c r="X8" s="27" t="str">
+        <v>498</v>
+      </c>
+      <c r="X8" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H8),H8/U8,"–")</f>
         <v>–</v>
       </c>
-      <c r="Y8" s="27" t="str">
+      <c r="Y8" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H8),H8/N8,"–")</f>
         <v>–</v>
       </c>
       <c r="Z8" s="6" t="s">
-        <v>378</v>
+        <v>499</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5355,85 +6503,85 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>379</v>
+        <v>500</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>380</v>
-      </c>
-      <c r="D9" s="22" t="n">
+        <v>501</v>
+      </c>
+      <c r="D9" s="23" t="n">
         <v>5.4</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24" t="s">
+      <c r="E9" s="24"/>
+      <c r="F9" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>381</v>
-      </c>
-      <c r="H9" s="25" t="str">
+        <v>502</v>
+      </c>
+      <c r="H9" s="26" t="str">
         <f aca="false">IF(E9="","Quote only",E9*INDEX(Assumptions!$B$12:$B$16,MATCH(F9,Assumptions!$A$12:$A$16,0)))</f>
         <v>Quote only</v>
       </c>
-      <c r="I9" s="25" t="str">
+      <c r="I9" s="26" t="str">
         <f aca="false">IF(ISNUMBER(H9),H9/D9,"–")</f>
         <v>–</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="K9" s="23" t="n">
+        <v>503</v>
+      </c>
+      <c r="K9" s="24" t="n">
         <v>105000</v>
       </c>
-      <c r="L9" s="23" t="n">
+      <c r="L9" s="24" t="n">
         <v>150000</v>
       </c>
-      <c r="M9" s="24" t="s">
+      <c r="M9" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N9" s="25" t="n">
+      <c r="N9" s="26" t="n">
         <f aca="false">AVERAGE(K9:L9)*INDEX(Assumptions!$B$12:$B$16,MATCH(M9,Assumptions!$A$12:$A$16,0))</f>
         <v>127500</v>
       </c>
-      <c r="O9" s="25" t="n">
+      <c r="O9" s="26" t="n">
         <f aca="false">N9/D9</f>
         <v>23611.1111111111</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>383</v>
+        <v>504</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="R9" s="23" t="n">
+        <v>505</v>
+      </c>
+      <c r="R9" s="24" t="n">
         <v>723</v>
       </c>
-      <c r="S9" s="23" t="n">
+      <c r="S9" s="24" t="n">
         <v>741</v>
       </c>
-      <c r="T9" s="24" t="s">
+      <c r="T9" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="U9" s="25" t="n">
+      <c r="U9" s="26" t="n">
         <f aca="false">AVERAGE(R9:S9)*INDEX(Assumptions!$B$12:$B$16,MATCH(T9,Assumptions!$A$12:$A$16,0))</f>
         <v>77218.8264</v>
       </c>
-      <c r="V9" s="25" t="n">
+      <c r="V9" s="26" t="n">
         <f aca="false">U9/D9</f>
         <v>14299.7826666667</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="X9" s="27" t="str">
+        <v>506</v>
+      </c>
+      <c r="X9" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H9),H9/U9,"–")</f>
         <v>–</v>
       </c>
-      <c r="Y9" s="27" t="str">
+      <c r="Y9" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H9),H9/N9,"–")</f>
         <v>–</v>
       </c>
       <c r="Z9" s="6" t="s">
-        <v>386</v>
+        <v>507</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5441,85 +6589,85 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>387</v>
+        <v>508</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="D10" s="22" t="n">
+        <v>509</v>
+      </c>
+      <c r="D10" s="23" t="n">
         <v>10.8</v>
       </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24" t="s">
+      <c r="E10" s="24"/>
+      <c r="F10" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>381</v>
-      </c>
-      <c r="H10" s="25" t="str">
+        <v>502</v>
+      </c>
+      <c r="H10" s="26" t="str">
         <f aca="false">IF(E10="","Quote only",E10*INDEX(Assumptions!$B$12:$B$16,MATCH(F10,Assumptions!$A$12:$A$16,0)))</f>
         <v>Quote only</v>
       </c>
-      <c r="I10" s="25" t="str">
+      <c r="I10" s="26" t="str">
         <f aca="false">IF(ISNUMBER(H10),H10/D10,"–")</f>
         <v>–</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="K10" s="23" t="n">
+        <v>510</v>
+      </c>
+      <c r="K10" s="24" t="n">
         <v>200000</v>
       </c>
-      <c r="L10" s="23" t="n">
+      <c r="L10" s="24" t="n">
         <v>290000</v>
       </c>
-      <c r="M10" s="24" t="s">
+      <c r="M10" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N10" s="25" t="n">
+      <c r="N10" s="26" t="n">
         <f aca="false">AVERAGE(K10:L10)*INDEX(Assumptions!$B$12:$B$16,MATCH(M10,Assumptions!$A$12:$A$16,0))</f>
         <v>245000</v>
       </c>
-      <c r="O10" s="25" t="n">
+      <c r="O10" s="26" t="n">
         <f aca="false">N10/D10</f>
         <v>22685.1851851852</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>383</v>
+        <v>504</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="R10" s="26" t="n">
+        <v>511</v>
+      </c>
+      <c r="R10" s="27" t="n">
         <v>1446</v>
       </c>
-      <c r="S10" s="26" t="n">
+      <c r="S10" s="27" t="n">
         <v>1482</v>
       </c>
-      <c r="T10" s="24" t="s">
+      <c r="T10" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="U10" s="25" t="n">
+      <c r="U10" s="26" t="n">
         <f aca="false">AVERAGE(R10:S10)*INDEX(Assumptions!$B$12:$B$16,MATCH(T10,Assumptions!$A$12:$A$16,0))</f>
         <v>154437.6528</v>
       </c>
-      <c r="V10" s="25" t="n">
+      <c r="V10" s="26" t="n">
         <f aca="false">U10/D10</f>
         <v>14299.7826666667</v>
       </c>
       <c r="W10" s="14" t="s">
-        <v>391</v>
-      </c>
-      <c r="X10" s="27" t="str">
+        <v>512</v>
+      </c>
+      <c r="X10" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H10),H10/U10,"–")</f>
         <v>–</v>
       </c>
-      <c r="Y10" s="27" t="str">
+      <c r="Y10" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H10),H10/N10,"–")</f>
         <v>–</v>
       </c>
       <c r="Z10" s="6" t="s">
-        <v>386</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5527,85 +6675,85 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>392</v>
+        <v>513</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24" t="s">
+      <c r="E11" s="24"/>
+      <c r="F11" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="H11" s="25" t="str">
+        <v>514</v>
+      </c>
+      <c r="H11" s="26" t="str">
         <f aca="false">IF(E11="","Quote only",E11*INDEX(Assumptions!$B$12:$B$16,MATCH(F11,Assumptions!$A$12:$A$16,0)))</f>
         <v>Quote only</v>
       </c>
-      <c r="I11" s="25" t="str">
+      <c r="I11" s="26" t="str">
         <f aca="false">IF(ISNUMBER(H11),H11/D11,"–")</f>
         <v>–</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="K11" s="23" t="n">
+        <v>515</v>
+      </c>
+      <c r="K11" s="24" t="n">
         <v>28000</v>
       </c>
-      <c r="L11" s="23" t="n">
+      <c r="L11" s="24" t="n">
         <v>32000</v>
       </c>
-      <c r="M11" s="24" t="s">
+      <c r="M11" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="N11" s="25" t="n">
+      <c r="N11" s="26" t="n">
         <f aca="false">AVERAGE(K11:L11)*INDEX(Assumptions!$B$12:$B$16,MATCH(M11,Assumptions!$A$12:$A$16,0))</f>
         <v>30000</v>
       </c>
-      <c r="O11" s="25" t="n">
+      <c r="O11" s="26" t="n">
         <f aca="false">N11/D11</f>
         <v>30000</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>395</v>
+        <v>516</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="R11" s="23" t="n">
+        <v>517</v>
+      </c>
+      <c r="R11" s="24" t="n">
         <v>70</v>
       </c>
-      <c r="S11" s="23" t="n">
+      <c r="S11" s="24" t="n">
         <v>90</v>
       </c>
-      <c r="T11" s="24" t="s">
+      <c r="T11" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="U11" s="25" t="n">
+      <c r="U11" s="26" t="n">
         <f aca="false">AVERAGE(R11:S11)*INDEX(Assumptions!$B$12:$B$16,MATCH(T11,Assumptions!$A$12:$A$16,0))</f>
         <v>7742.4</v>
       </c>
-      <c r="V11" s="25" t="n">
+      <c r="V11" s="26" t="n">
         <f aca="false">U11/D11</f>
         <v>7742.4</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>397</v>
-      </c>
-      <c r="X11" s="27" t="str">
+        <v>518</v>
+      </c>
+      <c r="X11" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H11),H11/U11,"–")</f>
         <v>–</v>
       </c>
-      <c r="Y11" s="27" t="str">
+      <c r="Y11" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H11),H11/N11,"–")</f>
         <v>–</v>
       </c>
       <c r="Z11" s="6" t="s">
-        <v>398</v>
+        <v>519</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5613,198 +6761,198 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>399</v>
+        <v>520</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>400</v>
-      </c>
-      <c r="D12" s="22" t="n">
+        <v>521</v>
+      </c>
+      <c r="D12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24" t="s">
+      <c r="E12" s="24"/>
+      <c r="F12" s="25" t="s">
         <v>54</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>401</v>
-      </c>
-      <c r="H12" s="25" t="str">
+        <v>522</v>
+      </c>
+      <c r="H12" s="26" t="str">
         <f aca="false">IF(E12="","Quote only",E12*INDEX(Assumptions!$B$12:$B$16,MATCH(F12,Assumptions!$A$12:$A$16,0)))</f>
         <v>Quote only</v>
       </c>
-      <c r="I12" s="25" t="str">
+      <c r="I12" s="26" t="str">
         <f aca="false">IF(ISNUMBER(H12),H12/D12,"–")</f>
         <v>–</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="K12" s="23" t="n">
+        <v>523</v>
+      </c>
+      <c r="K12" s="24" t="n">
         <v>55</v>
       </c>
-      <c r="L12" s="23" t="n">
+      <c r="L12" s="24" t="n">
         <v>75</v>
       </c>
-      <c r="M12" s="24" t="s">
+      <c r="M12" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="25" t="n">
+      <c r="N12" s="26" t="n">
         <f aca="false">AVERAGE(K12:L12)*INDEX(Assumptions!$B$12:$B$16,MATCH(M12,Assumptions!$A$12:$A$16,0))</f>
         <v>6290.7</v>
       </c>
-      <c r="O12" s="25" t="n">
+      <c r="O12" s="26" t="n">
         <f aca="false">N12/D12</f>
         <v>6290.7</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>403</v>
+        <v>524</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="R12" s="23" t="n">
+        <v>525</v>
+      </c>
+      <c r="R12" s="24" t="n">
         <v>360</v>
       </c>
-      <c r="S12" s="23" t="n">
+      <c r="S12" s="24" t="n">
         <v>443</v>
       </c>
-      <c r="T12" s="24" t="s">
+      <c r="T12" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="U12" s="25" t="n">
+      <c r="U12" s="26" t="n">
         <f aca="false">AVERAGE(R12:S12)*INDEX(Assumptions!$B$12:$B$16,MATCH(T12,Assumptions!$A$12:$A$16,0))</f>
         <v>5442.18067226891</v>
       </c>
-      <c r="V12" s="25" t="n">
+      <c r="V12" s="26" t="n">
         <f aca="false">U12/D12</f>
         <v>5442.18067226891</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>405</v>
-      </c>
-      <c r="X12" s="27" t="str">
+        <v>526</v>
+      </c>
+      <c r="X12" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H12),H12/U12,"–")</f>
         <v>–</v>
       </c>
-      <c r="Y12" s="27" t="str">
+      <c r="Y12" s="28" t="str">
         <f aca="false">IF(ISNUMBER(H12),H12/N12,"–")</f>
         <v>–</v>
       </c>
       <c r="Z12" s="6" t="s">
-        <v>406</v>
+        <v>527</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="28" t="s">
-        <v>407</v>
+      <c r="B14" s="29" t="s">
+        <v>528</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="19" t="s">
-        <v>408</v>
+        <v>529</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="19" t="s">
-        <v>409</v>
+        <v>530</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="19" t="s">
-        <v>410</v>
+        <v>531</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="19" t="s">
-        <v>411</v>
+        <v>532</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="10" t="s">
-        <v>412</v>
+        <v>533</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="29" t="s">
-        <v>341</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>348</v>
+      <c r="C22" s="30" t="s">
+        <v>462</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="C23" s="25" t="n">
+        <v>534</v>
+      </c>
+      <c r="C23" s="26" t="n">
         <f aca="false">O7</f>
         <v>21000</v>
       </c>
-      <c r="D23" s="25" t="n">
+      <c r="D23" s="26" t="n">
         <f aca="false">V7</f>
         <v>19356</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>414</v>
-      </c>
-      <c r="C24" s="25" t="n">
+        <v>535</v>
+      </c>
+      <c r="C24" s="26" t="n">
         <f aca="false">O9</f>
         <v>23611.1111111111</v>
       </c>
-      <c r="D24" s="25" t="n">
+      <c r="D24" s="26" t="n">
         <f aca="false">V9</f>
         <v>14299.7826666667</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>415</v>
-      </c>
-      <c r="C25" s="25" t="n">
+        <v>536</v>
+      </c>
+      <c r="C25" s="26" t="n">
         <f aca="false">O10</f>
         <v>22685.1851851852</v>
       </c>
-      <c r="D25" s="25" t="n">
+      <c r="D25" s="26" t="n">
         <f aca="false">V10</f>
         <v>14299.7826666667</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C26" s="25" t="n">
+        <v>537</v>
+      </c>
+      <c r="C26" s="26" t="n">
         <f aca="false">O11</f>
         <v>30000</v>
       </c>
-      <c r="D26" s="25" t="n">
+      <c r="D26" s="26" t="n">
         <f aca="false">V11</f>
         <v>7742.4</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>417</v>
-      </c>
-      <c r="C27" s="25" t="n">
+        <v>538</v>
+      </c>
+      <c r="C27" s="26" t="n">
         <f aca="false">O12</f>
         <v>6290.7</v>
       </c>
-      <c r="D27" s="25" t="n">
+      <c r="D27" s="26" t="n">
         <f aca="false">V12</f>
         <v>5442.18067226891</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="10" t="s">
-        <v>418</v>
-      </c>
-      <c r="C29" s="30" t="n">
+        <v>539</v>
+      </c>
+      <c r="C29" s="31" t="n">
         <f aca="false">I7</f>
         <v>268038.848</v>
       </c>
@@ -5821,7 +6969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -5840,20 +6988,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>419</v>
+        <v>540</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>420</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>421</v>
+        <v>542</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>422</v>
+        <v>543</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>3</v>
@@ -5862,13 +7010,13 @@
         <v>36</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>423</v>
+        <v>544</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>424</v>
+        <v>545</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>425</v>
+        <v>546</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>99</v>
@@ -5876,909 +7024,407 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>427</v>
-      </c>
-      <c r="C5" s="22" t="n">
+        <v>548</v>
+      </c>
+      <c r="C5" s="23" t="n">
         <v>0.365</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>428</v>
-      </c>
-      <c r="E5" s="31" t="n">
+        <v>549</v>
+      </c>
+      <c r="E5" s="32" t="n">
         <f aca="false">C5*1000*Assumptions!$B$15</f>
         <v>4947.43697478992</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>430</v>
+        <v>551</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>431</v>
+        <v>552</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="C6" s="22" t="n">
+        <v>553</v>
+      </c>
+      <c r="C6" s="23" t="n">
         <v>0.36</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>428</v>
-      </c>
-      <c r="E6" s="31" t="n">
+        <v>549</v>
+      </c>
+      <c r="E6" s="32" t="n">
         <f aca="false">C6*1000*Assumptions!$B$15</f>
         <v>4879.66386554622</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>433</v>
+        <v>554</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>434</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C7" s="22" t="n">
+        <v>556</v>
+      </c>
+      <c r="C7" s="23" t="n">
         <v>0.443</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>428</v>
-      </c>
-      <c r="E7" s="31" t="n">
+        <v>549</v>
+      </c>
+      <c r="E7" s="32" t="n">
         <f aca="false">C7*1000*Assumptions!$B$15</f>
         <v>6004.6974789916</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>433</v>
+        <v>554</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>434</v>
+        <v>555</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="C8" s="22" t="n">
+        <v>557</v>
+      </c>
+      <c r="C8" s="23" t="n">
         <v>0.49</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>428</v>
-      </c>
-      <c r="E8" s="31" t="n">
+        <v>549</v>
+      </c>
+      <c r="E8" s="32" t="n">
         <f aca="false">C8*1000*Assumptions!$B$15</f>
         <v>6641.76470588235</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>430</v>
+        <v>551</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>431</v>
+        <v>552</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="C9" s="32" t="n">
+        <v>558</v>
+      </c>
+      <c r="C9" s="33" t="n">
         <v>80</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E9" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E9" s="32" t="n">
         <f aca="false">C9*Assumptions!$B$13</f>
         <v>7742.4</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>439</v>
+        <v>560</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>440</v>
+        <v>561</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>441</v>
-      </c>
-      <c r="C10" s="32" t="n">
+        <v>562</v>
+      </c>
+      <c r="C10" s="33" t="n">
         <v>77</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E10" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E10" s="32" t="n">
         <f aca="false">C10*Assumptions!$B$13</f>
         <v>7452.06</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>442</v>
+        <v>563</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>443</v>
+        <v>564</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="C11" s="32" t="n">
+        <v>565</v>
+      </c>
+      <c r="C11" s="33" t="n">
         <v>66</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E11" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E11" s="32" t="n">
         <f aca="false">C11*Assumptions!$B$13</f>
         <v>6387.48</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>442</v>
+        <v>563</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>443</v>
+        <v>564</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>426</v>
+        <v>547</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>445</v>
-      </c>
-      <c r="C12" s="32" t="n">
+        <v>566</v>
+      </c>
+      <c r="C12" s="33" t="n">
         <v>140</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E12" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E12" s="32" t="n">
         <f aca="false">C12*Assumptions!$B$13</f>
         <v>13549.2</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>446</v>
+        <v>567</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>447</v>
+        <v>568</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>449</v>
-      </c>
-      <c r="C13" s="32" t="n">
+        <v>570</v>
+      </c>
+      <c r="C13" s="33" t="n">
         <v>72.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E13" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E13" s="32" t="n">
         <f aca="false">C13*Assumptions!$B$13</f>
         <v>7016.55</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>450</v>
+        <v>571</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>451</v>
+        <v>572</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>452</v>
-      </c>
-      <c r="C14" s="32" t="n">
+        <v>573</v>
+      </c>
+      <c r="C14" s="33" t="n">
         <v>57.5</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E14" s="31" t="n">
+        <v>559</v>
+      </c>
+      <c r="E14" s="32" t="n">
         <f aca="false">C14*Assumptions!$B$13</f>
         <v>5564.85</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>453</v>
+        <v>574</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>454</v>
+        <v>575</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>455</v>
-      </c>
-      <c r="C15" s="32" t="n">
+        <v>576</v>
+      </c>
+      <c r="C15" s="33" t="n">
         <v>27500</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>456</v>
-      </c>
-      <c r="E15" s="33" t="n">
+        <v>577</v>
+      </c>
+      <c r="E15" s="34" t="n">
         <f aca="false">C15</f>
         <v>27500</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>450</v>
+        <v>571</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>457</v>
+        <v>578</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="C16" s="32" t="n">
+        <v>579</v>
+      </c>
+      <c r="C16" s="33" t="n">
         <v>30000</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>456</v>
-      </c>
-      <c r="E16" s="33" t="n">
+        <v>577</v>
+      </c>
+      <c r="E16" s="34" t="n">
         <f aca="false">C16</f>
         <v>30000</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>429</v>
+        <v>550</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>450</v>
+        <v>571</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>459</v>
+        <v>580</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="C17" s="32" t="n">
+        <v>581</v>
+      </c>
+      <c r="C17" s="33" t="n">
         <v>285000</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="E17" s="33" t="n">
+        <v>582</v>
+      </c>
+      <c r="E17" s="34" t="n">
         <f aca="false">C17</f>
         <v>285000</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>462</v>
+        <v>583</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>463</v>
+        <v>584</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>464</v>
+        <v>585</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>465</v>
-      </c>
-      <c r="C18" s="32" t="n">
+        <v>586</v>
+      </c>
+      <c r="C18" s="33" t="n">
         <v>181000</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="E18" s="33" t="n">
+        <v>582</v>
+      </c>
+      <c r="E18" s="34" t="n">
         <f aca="false">C18</f>
         <v>181000</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>462</v>
+        <v>583</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>466</v>
+        <v>587</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>467</v>
+        <v>588</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>468</v>
-      </c>
-      <c r="C19" s="32" t="n">
+        <v>589</v>
+      </c>
+      <c r="C19" s="33" t="n">
         <v>148000</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="E19" s="33" t="n">
+        <v>582</v>
+      </c>
+      <c r="E19" s="34" t="n">
         <f aca="false">C19</f>
         <v>148000</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>462</v>
+        <v>583</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>469</v>
+        <v>590</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>470</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:C45"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="100"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
-        <v>471</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>472</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>474</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>475</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>477</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>479</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>481</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>484</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>488</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>490</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>496</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>497</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>501</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>505</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>507</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>509</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>515</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>517</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>518</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="C23" s="34" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
-        <v>523</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="C24" s="34" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>526</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>527</v>
-      </c>
-      <c r="C25" s="34" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>529</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>530</v>
-      </c>
-      <c r="C26" s="34" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>533</v>
-      </c>
-      <c r="C27" s="34" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>535</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>536</v>
-      </c>
-      <c r="C28" s="34" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>457</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>538</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>541</v>
-      </c>
-      <c r="C30" s="34" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="C31" s="34" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>547</v>
-      </c>
-      <c r="C32" s="34" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>549</v>
-      </c>
-      <c r="C33" s="34" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>551</v>
-      </c>
-      <c r="C34" s="34" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>443</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="C35" s="34" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>431</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>555</v>
-      </c>
-      <c r="C36" s="34" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>557</v>
-      </c>
-      <c r="C37" s="34" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>559</v>
-      </c>
-      <c r="C38" s="34" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
-        <v>454</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>561</v>
-      </c>
-      <c r="C39" s="34" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>563</v>
-      </c>
-      <c r="C40" s="34" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
-        <v>464</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>565</v>
-      </c>
-      <c r="C41" s="34" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="C42" s="34" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
-        <v>569</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>570</v>
-      </c>
-      <c r="C43" s="34" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
-        <v>447</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>572</v>
-      </c>
-      <c r="C44" s="34" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="C45" s="34" t="s">
-        <v>575</v>
+        <v>591</v>
       </c>
     </row>
   </sheetData>
@@ -6797,116 +7443,490 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>576</v>
+        <v>473</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>577</v>
+        <v>592</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>593</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>609</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="C16" s="35" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="C27" s="35" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="C28" s="35" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>578</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B29" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="C29" s="35" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="C30" s="35" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="C32" s="35" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
         <v>580</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>583</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>584</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="B33" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="C33" s="35" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="C35" s="35" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="C37" s="35" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="C38" s="35" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="C39" s="35" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>683</v>
+      </c>
+      <c r="C40" s="35" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="s">
         <v>585</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>586</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>587</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>588</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>589</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>590</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="B41" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="C41" s="35" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>592</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>593</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
-        <v>595</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>596</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>598</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>599</v>
+      <c r="B42" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="C43" s="35" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="C44" s="35" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>695</v>
       </c>
     </row>
   </sheetData>

</xml_diff>